<commit_message>
Add ITEM field to documents and rename STATUS DE CONTRATISTA label
- Nuevo campo ITEM en el registro de Documentos, despues de # TRANSMITTAL
  (importConfig, DOC_COLUMNS, columna item aditiva en init.sql).
- Etiqueta visible 'STATUS DE CONTRATISTA' renombrada a 'ESTATUS DE DOCUMENTO'
  (columna BD status_contratista sin cambios).
- Matriz de verificacion regenerada.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Cw5JMfxvGB8TrduB4fjsyK
</commit_message>
<xml_diff>
--- a/Matriz_Campos_ControlDoc.xlsx
+++ b/Matriz_Campos_ControlDoc.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:P1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -427,30 +427,33 @@
         <v># TRANSMITTAL</v>
       </c>
       <c r="I1" t="str">
+        <v>ITEM</v>
+      </c>
+      <c r="J1" t="str">
         <v>REFERENCIA</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>DOCUMENTO NRO</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>REV.</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>DESCRIPCIÓN</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>TIPO DE DOC</v>
       </c>
-      <c r="N1" t="str">
-        <v>STATUS DE CONTRATISTA</v>
-      </c>
       <c r="O1" t="str">
+        <v>ESTATUS DE DOCUMENTO</v>
+      </c>
+      <c r="P1" t="str">
         <v>RESPONSABLE</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -623,7 +626,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I69"/>
+  <dimension ref="A1:I70"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -894,10 +897,10 @@
         <v>9</v>
       </c>
       <c r="C10" t="str">
-        <v>REFERENCIA</v>
+        <v>ITEM</v>
       </c>
       <c r="D10" t="str">
-        <v>referencia</v>
+        <v>item</v>
       </c>
       <c r="E10" t="str">
         <v>texto</v>
@@ -923,16 +926,16 @@
         <v>10</v>
       </c>
       <c r="C11" t="str">
-        <v>DOCUMENTO NRO</v>
+        <v>REFERENCIA</v>
       </c>
       <c r="D11" t="str">
-        <v>documento_nro</v>
+        <v>referencia</v>
       </c>
       <c r="E11" t="str">
         <v>texto</v>
       </c>
       <c r="F11" t="str">
-        <v>SÍ</v>
+        <v/>
       </c>
       <c r="G11" t="str">
         <v/>
@@ -952,16 +955,16 @@
         <v>11</v>
       </c>
       <c r="C12" t="str">
-        <v>REV.</v>
+        <v>DOCUMENTO NRO</v>
       </c>
       <c r="D12" t="str">
-        <v>rev</v>
+        <v>documento_nro</v>
       </c>
       <c r="E12" t="str">
         <v>texto</v>
       </c>
       <c r="F12" t="str">
-        <v/>
+        <v>SÍ</v>
       </c>
       <c r="G12" t="str">
         <v/>
@@ -981,10 +984,10 @@
         <v>12</v>
       </c>
       <c r="C13" t="str">
-        <v>DESCRIPCIÓN</v>
+        <v>REV.</v>
       </c>
       <c r="D13" t="str">
-        <v>descripcion</v>
+        <v>rev</v>
       </c>
       <c r="E13" t="str">
         <v>texto</v>
@@ -1010,10 +1013,10 @@
         <v>13</v>
       </c>
       <c r="C14" t="str">
-        <v>TIPO DE DOC</v>
+        <v>DESCRIPCIÓN</v>
       </c>
       <c r="D14" t="str">
-        <v>tipo_doc</v>
+        <v>descripcion</v>
       </c>
       <c r="E14" t="str">
         <v>texto</v>
@@ -1039,10 +1042,10 @@
         <v>14</v>
       </c>
       <c r="C15" t="str">
-        <v>STATUS DE CONTRATISTA</v>
+        <v>TIPO DE DOC</v>
       </c>
       <c r="D15" t="str">
-        <v>status_contratista</v>
+        <v>tipo_doc</v>
       </c>
       <c r="E15" t="str">
         <v>texto</v>
@@ -1057,7 +1060,7 @@
         <v>columna real</v>
       </c>
       <c r="I15" t="str">
-        <v>APROBADO / EN REVISIÓN / CON OBSERVACIONES / ANULADO</v>
+        <v/>
       </c>
     </row>
     <row r="16">
@@ -1068,10 +1071,10 @@
         <v>15</v>
       </c>
       <c r="C16" t="str">
-        <v>RESPONSABLE</v>
+        <v>ESTATUS DE DOCUMENTO</v>
       </c>
       <c r="D16" t="str">
-        <v>responsable</v>
+        <v>status_contratista</v>
       </c>
       <c r="E16" t="str">
         <v>texto</v>
@@ -1086,65 +1089,65 @@
         <v>columna real</v>
       </c>
       <c r="I16" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>HOJA</v>
-      </c>
-      <c r="B18" t="str">
-        <v>ORDEN</v>
-      </c>
-      <c r="C18" t="str">
-        <v>ENCABEZADO EN EXCEL</v>
-      </c>
-      <c r="D18" t="str">
-        <v>CAMPO BD</v>
-      </c>
-      <c r="E18" t="str">
-        <v>TIPO</v>
-      </c>
-      <c r="F18" t="str">
-        <v>CLAVE ÚNICA</v>
-      </c>
-      <c r="G18" t="str">
-        <v>REQUERIDO</v>
-      </c>
-      <c r="H18" t="str">
-        <v>DESTINO</v>
-      </c>
-      <c r="I18" t="str">
-        <v>NOTAS</v>
+        <v>Antes "STATUS DE CONTRATISTA". Columna BD: status_contratista. APROBADO / EN REVISIÓN / CON OBSERVACIONES / ANULADO</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Documentos</v>
+      </c>
+      <c r="B17">
+        <v>16</v>
+      </c>
+      <c r="C17" t="str">
+        <v>RESPONSABLE</v>
+      </c>
+      <c r="D17" t="str">
+        <v>responsable</v>
+      </c>
+      <c r="E17" t="str">
+        <v>texto</v>
+      </c>
+      <c r="F17" t="str">
+        <v/>
+      </c>
+      <c r="G17" t="str">
+        <v/>
+      </c>
+      <c r="H17" t="str">
+        <v>columna real</v>
+      </c>
+      <c r="I17" t="str">
+        <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Contratos</v>
-      </c>
-      <c r="B19">
-        <v>1</v>
+        <v>HOJA</v>
+      </c>
+      <c r="B19" t="str">
+        <v>ORDEN</v>
       </c>
       <c r="C19" t="str">
-        <v>CLASE CONTRATO</v>
+        <v>ENCABEZADO EN EXCEL</v>
       </c>
       <c r="D19" t="str">
-        <v>type</v>
+        <v>CAMPO BD</v>
       </c>
       <c r="E19" t="str">
-        <v>texto</v>
+        <v>TIPO</v>
       </c>
       <c r="F19" t="str">
-        <v/>
+        <v>CLAVE ÚNICA</v>
       </c>
       <c r="G19" t="str">
-        <v/>
+        <v>REQUERIDO</v>
       </c>
       <c r="H19" t="str">
-        <v>columna real</v>
+        <v>DESTINO</v>
       </c>
       <c r="I19" t="str">
-        <v/>
+        <v>NOTAS</v>
       </c>
     </row>
     <row r="20">
@@ -1152,13 +1155,13 @@
         <v>Contratos</v>
       </c>
       <c r="B20">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C20" t="str">
-        <v>Tipo Inversion</v>
+        <v>CLASE CONTRATO</v>
       </c>
       <c r="D20" t="str">
-        <v>(extra_data)</v>
+        <v>type</v>
       </c>
       <c r="E20" t="str">
         <v>texto</v>
@@ -1170,7 +1173,7 @@
         <v/>
       </c>
       <c r="H20" t="str">
-        <v>extra_data (JSON)</v>
+        <v>columna real</v>
       </c>
       <c r="I20" t="str">
         <v/>
@@ -1181,10 +1184,10 @@
         <v>Contratos</v>
       </c>
       <c r="B21">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C21" t="str">
-        <v>Consultoria</v>
+        <v>Tipo Inversion</v>
       </c>
       <c r="D21" t="str">
         <v>(extra_data)</v>
@@ -1210,13 +1213,13 @@
         <v>Contratos</v>
       </c>
       <c r="B22">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C22" t="str">
-        <v>ESTADO</v>
+        <v>Consultoria</v>
       </c>
       <c r="D22" t="str">
-        <v>status</v>
+        <v>(extra_data)</v>
       </c>
       <c r="E22" t="str">
         <v>texto</v>
@@ -1228,7 +1231,7 @@
         <v/>
       </c>
       <c r="H22" t="str">
-        <v>columna real</v>
+        <v>extra_data (JSON)</v>
       </c>
       <c r="I22" t="str">
         <v/>
@@ -1239,13 +1242,13 @@
         <v>Contratos</v>
       </c>
       <c r="B23">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C23" t="str">
-        <v>A SAP Reg</v>
+        <v>ESTADO</v>
       </c>
       <c r="D23" t="str">
-        <v>(extra_data)</v>
+        <v>status</v>
       </c>
       <c r="E23" t="str">
         <v>texto</v>
@@ -1257,7 +1260,7 @@
         <v/>
       </c>
       <c r="H23" t="str">
-        <v>extra_data (JSON)</v>
+        <v>columna real</v>
       </c>
       <c r="I23" t="str">
         <v/>
@@ -1268,10 +1271,10 @@
         <v>Contratos</v>
       </c>
       <c r="B24">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C24" t="str">
-        <v>Estado Contrato SAP</v>
+        <v>A SAP Reg</v>
       </c>
       <c r="D24" t="str">
         <v>(extra_data)</v>
@@ -1297,10 +1300,10 @@
         <v>Contratos</v>
       </c>
       <c r="B25">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C25" t="str">
-        <v>B Custodia</v>
+        <v>Estado Contrato SAP</v>
       </c>
       <c r="D25" t="str">
         <v>(extra_data)</v>
@@ -1326,10 +1329,10 @@
         <v>Contratos</v>
       </c>
       <c r="B26">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C26" t="str">
-        <v>C OS(F=OK)</v>
+        <v>B Custodia</v>
       </c>
       <c r="D26" t="str">
         <v>(extra_data)</v>
@@ -1355,10 +1358,10 @@
         <v>Contratos</v>
       </c>
       <c r="B27">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C27" t="str">
-        <v>Estado OS SAP</v>
+        <v>C OS(F=OK)</v>
       </c>
       <c r="D27" t="str">
         <v>(extra_data)</v>
@@ -1384,10 +1387,10 @@
         <v>Contratos</v>
       </c>
       <c r="B28">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C28" t="str">
-        <v>RESPONSABLE</v>
+        <v>Estado OS SAP</v>
       </c>
       <c r="D28" t="str">
         <v>(extra_data)</v>
@@ -1413,10 +1416,10 @@
         <v>Contratos</v>
       </c>
       <c r="B29">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C29" t="str">
-        <v>GRUPO INVERSION</v>
+        <v>RESPONSABLE</v>
       </c>
       <c r="D29" t="str">
         <v>(extra_data)</v>
@@ -1442,10 +1445,10 @@
         <v>Contratos</v>
       </c>
       <c r="B30">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C30" t="str">
-        <v>AREA SOLICITANTE</v>
+        <v>GRUPO INVERSION</v>
       </c>
       <c r="D30" t="str">
         <v>(extra_data)</v>
@@ -1471,10 +1474,10 @@
         <v>Contratos</v>
       </c>
       <c r="B31">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C31" t="str">
-        <v>COD INVERSION</v>
+        <v>AREA SOLICITANTE</v>
       </c>
       <c r="D31" t="str">
         <v>(extra_data)</v>
@@ -1500,10 +1503,10 @@
         <v>Contratos</v>
       </c>
       <c r="B32">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C32" t="str">
-        <v>CC</v>
+        <v>COD INVERSION</v>
       </c>
       <c r="D32" t="str">
         <v>(extra_data)</v>
@@ -1529,10 +1532,10 @@
         <v>Contratos</v>
       </c>
       <c r="B33">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C33" t="str">
-        <v>CIRCUITO</v>
+        <v>CC</v>
       </c>
       <c r="D33" t="str">
         <v>(extra_data)</v>
@@ -1558,10 +1561,10 @@
         <v>Contratos</v>
       </c>
       <c r="B34">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C34" t="str">
-        <v>MODALIDAD CONTRATACION</v>
+        <v>CIRCUITO</v>
       </c>
       <c r="D34" t="str">
         <v>(extra_data)</v>
@@ -1587,10 +1590,10 @@
         <v>Contratos</v>
       </c>
       <c r="B35">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C35" t="str">
-        <v>Condiciones (Adel, % Ret FG, Ret FC)</v>
+        <v>MODALIDAD CONTRATACION</v>
       </c>
       <c r="D35" t="str">
         <v>(extra_data)</v>
@@ -1616,16 +1619,16 @@
         <v>Contratos</v>
       </c>
       <c r="B36">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C36" t="str">
-        <v>FECHA SUSCRIPCIÓN DE CONTRATO</v>
+        <v>Condiciones (Adel, % Ret FG, Ret FC)</v>
       </c>
       <c r="D36" t="str">
-        <v>start_date</v>
+        <v>(extra_data)</v>
       </c>
       <c r="E36" t="str">
-        <v>fecha</v>
+        <v>texto</v>
       </c>
       <c r="F36" t="str">
         <v/>
@@ -1634,7 +1637,7 @@
         <v/>
       </c>
       <c r="H36" t="str">
-        <v>columna real</v>
+        <v>extra_data (JSON)</v>
       </c>
       <c r="I36" t="str">
         <v/>
@@ -1645,13 +1648,13 @@
         <v>Contratos</v>
       </c>
       <c r="B37">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C37" t="str">
-        <v>FIN VIGENCIA CONTRATO</v>
+        <v>FECHA SUSCRIPCIÓN DE CONTRATO</v>
       </c>
       <c r="D37" t="str">
-        <v>end_date</v>
+        <v>start_date</v>
       </c>
       <c r="E37" t="str">
         <v>fecha</v>
@@ -1674,16 +1677,16 @@
         <v>Contratos</v>
       </c>
       <c r="B38">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C38" t="str">
-        <v>Fecha Acta de entrega de terreno</v>
+        <v>FIN VIGENCIA CONTRATO</v>
       </c>
       <c r="D38" t="str">
-        <v>(extra_data)</v>
+        <v>end_date</v>
       </c>
       <c r="E38" t="str">
-        <v>texto</v>
+        <v>fecha</v>
       </c>
       <c r="F38" t="str">
         <v/>
@@ -1692,7 +1695,7 @@
         <v/>
       </c>
       <c r="H38" t="str">
-        <v>extra_data (JSON)</v>
+        <v>columna real</v>
       </c>
       <c r="I38" t="str">
         <v/>
@@ -1703,10 +1706,10 @@
         <v>Contratos</v>
       </c>
       <c r="B39">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C39" t="str">
-        <v>Fecha Acta de INICIO DE OBRA2</v>
+        <v>Fecha Acta de entrega de terreno</v>
       </c>
       <c r="D39" t="str">
         <v>(extra_data)</v>
@@ -1732,10 +1735,10 @@
         <v>Contratos</v>
       </c>
       <c r="B40">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C40" t="str">
-        <v>PLAZO DE EJECUCION / FABRICACION</v>
+        <v>Fecha Acta de INICIO DE OBRA2</v>
       </c>
       <c r="D40" t="str">
         <v>(extra_data)</v>
@@ -1761,10 +1764,10 @@
         <v>Contratos</v>
       </c>
       <c r="B41">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C41" t="str">
-        <v>Fecha termino según contrato</v>
+        <v>PLAZO DE EJECUCION / FABRICACION</v>
       </c>
       <c r="D41" t="str">
         <v>(extra_data)</v>
@@ -1790,10 +1793,10 @@
         <v>Contratos</v>
       </c>
       <c r="B42">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C42" t="str">
-        <v>Z Ampliación de plazo</v>
+        <v>Fecha termino según contrato</v>
       </c>
       <c r="D42" t="str">
         <v>(extra_data)</v>
@@ -1819,10 +1822,10 @@
         <v>Contratos</v>
       </c>
       <c r="B43">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C43" t="str">
-        <v>Plazo penalizado</v>
+        <v>Z Ampliación de plazo</v>
       </c>
       <c r="D43" t="str">
         <v>(extra_data)</v>
@@ -1848,10 +1851,10 @@
         <v>Contratos</v>
       </c>
       <c r="B44">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C44" t="str">
-        <v>Plazo de Ejecucion ajustado</v>
+        <v>Plazo penalizado</v>
       </c>
       <c r="D44" t="str">
         <v>(extra_data)</v>
@@ -1877,10 +1880,10 @@
         <v>Contratos</v>
       </c>
       <c r="B45">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C45" t="str">
-        <v>Plazo total</v>
+        <v>Plazo de Ejecucion ajustado</v>
       </c>
       <c r="D45" t="str">
         <v>(extra_data)</v>
@@ -1906,10 +1909,10 @@
         <v>Contratos</v>
       </c>
       <c r="B46">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C46" t="str">
-        <v>Fecha Recepción Provisional / Fin según contrato (Ultima)</v>
+        <v>Plazo total</v>
       </c>
       <c r="D46" t="str">
         <v>(extra_data)</v>
@@ -1935,16 +1938,16 @@
         <v>Contratos</v>
       </c>
       <c r="B47">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C47" t="str">
-        <v>Fecha Recepcion Final</v>
+        <v>Fecha Recepción Provisional / Fin según contrato (Ultima)</v>
       </c>
       <c r="D47" t="str">
-        <v>actual_end_date</v>
+        <v>(extra_data)</v>
       </c>
       <c r="E47" t="str">
-        <v>fecha</v>
+        <v>texto</v>
       </c>
       <c r="F47" t="str">
         <v/>
@@ -1953,7 +1956,7 @@
         <v/>
       </c>
       <c r="H47" t="str">
-        <v>columna real</v>
+        <v>extra_data (JSON)</v>
       </c>
       <c r="I47" t="str">
         <v/>
@@ -1964,16 +1967,16 @@
         <v>Contratos</v>
       </c>
       <c r="B48">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C48" t="str">
-        <v>Plazo de garantia</v>
+        <v>Fecha Recepcion Final</v>
       </c>
       <c r="D48" t="str">
-        <v>(extra_data)</v>
+        <v>actual_end_date</v>
       </c>
       <c r="E48" t="str">
-        <v>texto</v>
+        <v>fecha</v>
       </c>
       <c r="F48" t="str">
         <v/>
@@ -1982,7 +1985,7 @@
         <v/>
       </c>
       <c r="H48" t="str">
-        <v>extra_data (JSON)</v>
+        <v>columna real</v>
       </c>
       <c r="I48" t="str">
         <v/>
@@ -1993,10 +1996,10 @@
         <v>Contratos</v>
       </c>
       <c r="B49">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C49" t="str">
-        <v>Inicio de operación del PYT</v>
+        <v>Plazo de garantia</v>
       </c>
       <c r="D49" t="str">
         <v>(extra_data)</v>
@@ -2022,10 +2025,10 @@
         <v>Contratos</v>
       </c>
       <c r="B50">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C50" t="str">
-        <v>Por Pagar Garantia (Cuenta 30 dias antes Venc.)</v>
+        <v>Inicio de operación del PYT</v>
       </c>
       <c r="D50" t="str">
         <v>(extra_data)</v>
@@ -2051,10 +2054,10 @@
         <v>Contratos</v>
       </c>
       <c r="B51">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C51" t="str">
-        <v>ID</v>
+        <v>Por Pagar Garantia (Cuenta 30 dias antes Venc.)</v>
       </c>
       <c r="D51" t="str">
         <v>(extra_data)</v>
@@ -2080,25 +2083,25 @@
         <v>Contratos</v>
       </c>
       <c r="B52">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C52" t="str">
-        <v>N° CONTRATO</v>
+        <v>ID</v>
       </c>
       <c r="D52" t="str">
-        <v>code</v>
+        <v>(extra_data)</v>
       </c>
       <c r="E52" t="str">
         <v>texto</v>
       </c>
       <c r="F52" t="str">
-        <v>SÍ</v>
+        <v/>
       </c>
       <c r="G52" t="str">
-        <v>SÍ</v>
+        <v/>
       </c>
       <c r="H52" t="str">
-        <v>columna real</v>
+        <v>extra_data (JSON)</v>
       </c>
       <c r="I52" t="str">
         <v/>
@@ -2109,25 +2112,25 @@
         <v>Contratos</v>
       </c>
       <c r="B53">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C53" t="str">
-        <v>CONTRATO DWH</v>
+        <v>N° CONTRATO</v>
       </c>
       <c r="D53" t="str">
-        <v>(extra_data)</v>
+        <v>code</v>
       </c>
       <c r="E53" t="str">
         <v>texto</v>
       </c>
       <c r="F53" t="str">
-        <v/>
+        <v>SÍ</v>
       </c>
       <c r="G53" t="str">
-        <v/>
+        <v>SÍ</v>
       </c>
       <c r="H53" t="str">
-        <v>extra_data (JSON)</v>
+        <v>columna real</v>
       </c>
       <c r="I53" t="str">
         <v/>
@@ -2138,10 +2141,10 @@
         <v>Contratos</v>
       </c>
       <c r="B54">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C54" t="str">
-        <v>ADENDA</v>
+        <v>CONTRATO DWH</v>
       </c>
       <c r="D54" t="str">
         <v>(extra_data)</v>
@@ -2167,10 +2170,10 @@
         <v>Contratos</v>
       </c>
       <c r="B55">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C55" t="str">
-        <v>RUC</v>
+        <v>ADENDA</v>
       </c>
       <c r="D55" t="str">
         <v>(extra_data)</v>
@@ -2196,10 +2199,10 @@
         <v>Contratos</v>
       </c>
       <c r="B56">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C56" t="str">
-        <v>EMPRESA</v>
+        <v>RUC</v>
       </c>
       <c r="D56" t="str">
         <v>(extra_data)</v>
@@ -2225,13 +2228,13 @@
         <v>Contratos</v>
       </c>
       <c r="B57">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C57" t="str">
-        <v>DESCRIPCION CONTRATO</v>
+        <v>EMPRESA</v>
       </c>
       <c r="D57" t="str">
-        <v>title</v>
+        <v>(extra_data)</v>
       </c>
       <c r="E57" t="str">
         <v>texto</v>
@@ -2240,10 +2243,10 @@
         <v/>
       </c>
       <c r="G57" t="str">
-        <v>SÍ</v>
+        <v/>
       </c>
       <c r="H57" t="str">
-        <v>columna real</v>
+        <v>extra_data (JSON)</v>
       </c>
       <c r="I57" t="str">
         <v/>
@@ -2254,13 +2257,13 @@
         <v>Contratos</v>
       </c>
       <c r="B58">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C58" t="str">
-        <v>Contrato en Chino</v>
+        <v>DESCRIPCION CONTRATO</v>
       </c>
       <c r="D58" t="str">
-        <v>(extra_data)</v>
+        <v>title</v>
       </c>
       <c r="E58" t="str">
         <v>texto</v>
@@ -2269,10 +2272,10 @@
         <v/>
       </c>
       <c r="G58" t="str">
-        <v/>
+        <v>SÍ</v>
       </c>
       <c r="H58" t="str">
-        <v>extra_data (JSON)</v>
+        <v>columna real</v>
       </c>
       <c r="I58" t="str">
         <v/>
@@ -2283,10 +2286,10 @@
         <v>Contratos</v>
       </c>
       <c r="B59">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C59" t="str">
-        <v>NOMBRE ESPECIFICO</v>
+        <v>Contrato en Chino</v>
       </c>
       <c r="D59" t="str">
         <v>(extra_data)</v>
@@ -2312,10 +2315,10 @@
         <v>Contratos</v>
       </c>
       <c r="B60">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C60" t="str">
-        <v>DESCRIPCION DE LA ADENDA</v>
+        <v>NOMBRE ESPECIFICO</v>
       </c>
       <c r="D60" t="str">
         <v>(extra_data)</v>
@@ -2341,10 +2344,10 @@
         <v>Contratos</v>
       </c>
       <c r="B61">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C61" t="str">
-        <v>CONTRATO_</v>
+        <v>DESCRIPCION DE LA ADENDA</v>
       </c>
       <c r="D61" t="str">
         <v>(extra_data)</v>
@@ -2370,10 +2373,10 @@
         <v>Contratos</v>
       </c>
       <c r="B62">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C62" t="str">
-        <v>EMPRESA_</v>
+        <v>CONTRATO_</v>
       </c>
       <c r="D62" t="str">
         <v>(extra_data)</v>
@@ -2399,10 +2402,10 @@
         <v>Contratos</v>
       </c>
       <c r="B63">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C63" t="str">
-        <v>CONTRATO_ NOMBRE INFORME</v>
+        <v>EMPRESA_</v>
       </c>
       <c r="D63" t="str">
         <v>(extra_data)</v>
@@ -2428,13 +2431,13 @@
         <v>Contratos</v>
       </c>
       <c r="B64">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C64" t="str">
-        <v>MONEDA</v>
+        <v>CONTRATO_ NOMBRE INFORME</v>
       </c>
       <c r="D64" t="str">
-        <v>currency</v>
+        <v>(extra_data)</v>
       </c>
       <c r="E64" t="str">
         <v>texto</v>
@@ -2446,7 +2449,7 @@
         <v/>
       </c>
       <c r="H64" t="str">
-        <v>columna real</v>
+        <v>extra_data (JSON)</v>
       </c>
       <c r="I64" t="str">
         <v/>
@@ -2457,16 +2460,16 @@
         <v>Contratos</v>
       </c>
       <c r="B65">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C65" t="str">
-        <v>PPTO BASE</v>
+        <v>MONEDA</v>
       </c>
       <c r="D65" t="str">
-        <v>(extra_data)</v>
+        <v>currency</v>
       </c>
       <c r="E65" t="str">
-        <v>numero</v>
+        <v>texto</v>
       </c>
       <c r="F65" t="str">
         <v/>
@@ -2475,7 +2478,7 @@
         <v/>
       </c>
       <c r="H65" t="str">
-        <v>extra_data (JSON)</v>
+        <v>columna real</v>
       </c>
       <c r="I65" t="str">
         <v/>
@@ -2486,10 +2489,10 @@
         <v>Contratos</v>
       </c>
       <c r="B66">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C66" t="str">
-        <v>MONTO CONTRATADO S/ (SIN IGV)</v>
+        <v>PPTO BASE</v>
       </c>
       <c r="D66" t="str">
         <v>(extra_data)</v>
@@ -2515,10 +2518,10 @@
         <v>Contratos</v>
       </c>
       <c r="B67">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C67" t="str">
-        <v>MONTO CONTRATADO US$ (SIN IGV)</v>
+        <v>MONTO CONTRATADO S/ (SIN IGV)</v>
       </c>
       <c r="D67" t="str">
         <v>(extra_data)</v>
@@ -2544,10 +2547,10 @@
         <v>Contratos</v>
       </c>
       <c r="B68">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C68" t="str">
-        <v>MONTO CONTRATADO S/ (CON IGV)</v>
+        <v>MONTO CONTRATADO US$ (SIN IGV)</v>
       </c>
       <c r="D68" t="str">
         <v>(extra_data)</v>
@@ -2573,10 +2576,10 @@
         <v>Contratos</v>
       </c>
       <c r="B69">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C69" t="str">
-        <v>MONTO CONTRATADO US$ (CON IGV)</v>
+        <v>MONTO CONTRATADO S/ (CON IGV)</v>
       </c>
       <c r="D69" t="str">
         <v>(extra_data)</v>
@@ -2597,9 +2600,38 @@
         <v/>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>Contratos</v>
+      </c>
+      <c r="B70">
+        <v>51</v>
+      </c>
+      <c r="C70" t="str">
+        <v>MONTO CONTRATADO US$ (CON IGV)</v>
+      </c>
+      <c r="D70" t="str">
+        <v>(extra_data)</v>
+      </c>
+      <c r="E70" t="str">
+        <v>numero</v>
+      </c>
+      <c r="F70" t="str">
+        <v/>
+      </c>
+      <c r="G70" t="str">
+        <v/>
+      </c>
+      <c r="H70" t="str">
+        <v>extra_data (JSON)</v>
+      </c>
+      <c r="I70" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I69"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I70"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Renombrar campos de Documentos y agregar RUC
Renombra las etiquetas de la grilla de Documentos y los encabezados del
Excel de sincronización (las columnas en BD no cambian):
- STATUS -> TIPO DE FLUJO (columna BD: status)
- STATUS G -> ESTADO TRANSMITTAL (columna BD: status_g)
- CONTRATO -> CONTRATO DC (columna BD: contrato)

Agrega el nuevo campo RUC (columna BD documents.ruc, encabezado "RUC").

El mapeo del Excel conserva los encabezados antiguos como alias para no
romper hojas existentes. Actualiza importConfig, syncDocuments, route de
documentos, init.sql, la matriz de campos, DocumentDetail, el reporte de
presentación y la documentación.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DNHZcSw8XiavXpJ1rPNtEg
</commit_message>
<xml_diff>
--- a/Matriz_Campos_ControlDoc.xlsx
+++ b/Matriz_Campos_ControlDoc.xlsx
@@ -399,14 +399,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:Q1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>STATUS</v>
+        <v>TIPO DE FLUJO</v>
       </c>
       <c r="B1" t="str">
-        <v>STATUS G</v>
+        <v>ESTADO TRANSMITTAL</v>
       </c>
       <c r="C1" t="str">
         <v>N° CONTRATO</v>
@@ -415,45 +415,48 @@
         <v>EMPRESA</v>
       </c>
       <c r="E1" t="str">
-        <v>CONTRATO</v>
+        <v>RUC</v>
       </c>
       <c r="F1" t="str">
+        <v>CONTRATO DC</v>
+      </c>
+      <c r="G1" t="str">
         <v>DESCRIPCIÓN CONTRATO</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>FECHA</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v># TRANSMITTAL</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>ITEM</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>REFERENCIA</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>DOCUMENTO NRO</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>REV.</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>DESCRIPCIÓN</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>TIPO DE DOC</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>ESTATUS DE DOCUMENTO</v>
       </c>
-      <c r="P1" t="str">
+      <c r="Q1" t="str">
         <v>RESPONSABLE</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -626,7 +629,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I70"/>
+  <dimension ref="A1:I71"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -665,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="C2" t="str">
-        <v>STATUS</v>
+        <v>TIPO DE FLUJO</v>
       </c>
       <c r="D2" t="str">
         <v>status</v>
@@ -683,7 +686,7 @@
         <v>columna real</v>
       </c>
       <c r="I2" t="str">
-        <v>ENVIADO / RECIBIDO (del transmittal)</v>
+        <v>Antes "STATUS". Columna BD: status. ENVIADO / RECIBIDO (del transmittal)</v>
       </c>
     </row>
     <row r="3">
@@ -694,7 +697,7 @@
         <v>2</v>
       </c>
       <c r="C3" t="str">
-        <v>STATUS G</v>
+        <v>ESTADO TRANSMITTAL</v>
       </c>
       <c r="D3" t="str">
         <v>status_g</v>
@@ -712,7 +715,7 @@
         <v>columna real</v>
       </c>
       <c r="I3" t="str">
-        <v>ATENDIDO / PENDIENTE (atención)</v>
+        <v>Antes "STATUS G". Columna BD: status_g. ATENDIDO / PENDIENTE (atención)</v>
       </c>
     </row>
     <row r="4">
@@ -781,10 +784,10 @@
         <v>5</v>
       </c>
       <c r="C6" t="str">
-        <v>CONTRATO</v>
+        <v>RUC</v>
       </c>
       <c r="D6" t="str">
-        <v>contrato</v>
+        <v>ruc</v>
       </c>
       <c r="E6" t="str">
         <v>texto</v>
@@ -799,7 +802,7 @@
         <v>columna real</v>
       </c>
       <c r="I6" t="str">
-        <v/>
+        <v>RUC de la empresa</v>
       </c>
     </row>
     <row r="7">
@@ -810,10 +813,10 @@
         <v>6</v>
       </c>
       <c r="C7" t="str">
-        <v>DESCRIPCIÓN CONTRATO</v>
+        <v>CONTRATO DC</v>
       </c>
       <c r="D7" t="str">
-        <v>descripcion_contrato</v>
+        <v>contrato</v>
       </c>
       <c r="E7" t="str">
         <v>texto</v>
@@ -828,7 +831,7 @@
         <v>columna real</v>
       </c>
       <c r="I7" t="str">
-        <v/>
+        <v>Antes "CONTRATO". Columna BD: contrato</v>
       </c>
     </row>
     <row r="8">
@@ -839,13 +842,13 @@
         <v>7</v>
       </c>
       <c r="C8" t="str">
-        <v>FECHA</v>
+        <v>DESCRIPCIÓN CONTRATO</v>
       </c>
       <c r="D8" t="str">
-        <v>fecha</v>
+        <v>descripcion_contrato</v>
       </c>
       <c r="E8" t="str">
-        <v>fecha</v>
+        <v>texto</v>
       </c>
       <c r="F8" t="str">
         <v/>
@@ -868,16 +871,16 @@
         <v>8</v>
       </c>
       <c r="C9" t="str">
-        <v># TRANSMITTAL</v>
+        <v>FECHA</v>
       </c>
       <c r="D9" t="str">
-        <v>transmittal</v>
+        <v>fecha</v>
       </c>
       <c r="E9" t="str">
-        <v>texto</v>
+        <v>fecha</v>
       </c>
       <c r="F9" t="str">
-        <v>SÍ</v>
+        <v/>
       </c>
       <c r="G9" t="str">
         <v/>
@@ -897,16 +900,16 @@
         <v>9</v>
       </c>
       <c r="C10" t="str">
-        <v>ITEM</v>
+        <v># TRANSMITTAL</v>
       </c>
       <c r="D10" t="str">
-        <v>item</v>
+        <v>transmittal</v>
       </c>
       <c r="E10" t="str">
         <v>texto</v>
       </c>
       <c r="F10" t="str">
-        <v/>
+        <v>SÍ</v>
       </c>
       <c r="G10" t="str">
         <v/>
@@ -926,10 +929,10 @@
         <v>10</v>
       </c>
       <c r="C11" t="str">
-        <v>REFERENCIA</v>
+        <v>ITEM</v>
       </c>
       <c r="D11" t="str">
-        <v>referencia</v>
+        <v>item</v>
       </c>
       <c r="E11" t="str">
         <v>texto</v>
@@ -955,16 +958,16 @@
         <v>11</v>
       </c>
       <c r="C12" t="str">
-        <v>DOCUMENTO NRO</v>
+        <v>REFERENCIA</v>
       </c>
       <c r="D12" t="str">
-        <v>documento_nro</v>
+        <v>referencia</v>
       </c>
       <c r="E12" t="str">
         <v>texto</v>
       </c>
       <c r="F12" t="str">
-        <v>SÍ</v>
+        <v/>
       </c>
       <c r="G12" t="str">
         <v/>
@@ -984,16 +987,16 @@
         <v>12</v>
       </c>
       <c r="C13" t="str">
-        <v>REV.</v>
+        <v>DOCUMENTO NRO</v>
       </c>
       <c r="D13" t="str">
-        <v>rev</v>
+        <v>documento_nro</v>
       </c>
       <c r="E13" t="str">
         <v>texto</v>
       </c>
       <c r="F13" t="str">
-        <v/>
+        <v>SÍ</v>
       </c>
       <c r="G13" t="str">
         <v/>
@@ -1013,10 +1016,10 @@
         <v>13</v>
       </c>
       <c r="C14" t="str">
-        <v>DESCRIPCIÓN</v>
+        <v>REV.</v>
       </c>
       <c r="D14" t="str">
-        <v>descripcion</v>
+        <v>rev</v>
       </c>
       <c r="E14" t="str">
         <v>texto</v>
@@ -1042,10 +1045,10 @@
         <v>14</v>
       </c>
       <c r="C15" t="str">
-        <v>TIPO DE DOC</v>
+        <v>DESCRIPCIÓN</v>
       </c>
       <c r="D15" t="str">
-        <v>tipo_doc</v>
+        <v>descripcion</v>
       </c>
       <c r="E15" t="str">
         <v>texto</v>
@@ -1071,10 +1074,10 @@
         <v>15</v>
       </c>
       <c r="C16" t="str">
-        <v>ESTATUS DE DOCUMENTO</v>
+        <v>TIPO DE DOC</v>
       </c>
       <c r="D16" t="str">
-        <v>status_contratista</v>
+        <v>tipo_doc</v>
       </c>
       <c r="E16" t="str">
         <v>texto</v>
@@ -1089,7 +1092,7 @@
         <v>columna real</v>
       </c>
       <c r="I16" t="str">
-        <v>Antes "STATUS DE CONTRATISTA". Columna BD: status_contratista. APROBADO / EN REVISIÓN / CON OBSERVACIONES / ANULADO</v>
+        <v/>
       </c>
     </row>
     <row r="17">
@@ -1100,10 +1103,10 @@
         <v>16</v>
       </c>
       <c r="C17" t="str">
-        <v>RESPONSABLE</v>
+        <v>ESTATUS DE DOCUMENTO</v>
       </c>
       <c r="D17" t="str">
-        <v>responsable</v>
+        <v>status_contratista</v>
       </c>
       <c r="E17" t="str">
         <v>texto</v>
@@ -1118,65 +1121,65 @@
         <v>columna real</v>
       </c>
       <c r="I17" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>HOJA</v>
-      </c>
-      <c r="B19" t="str">
-        <v>ORDEN</v>
-      </c>
-      <c r="C19" t="str">
-        <v>ENCABEZADO EN EXCEL</v>
-      </c>
-      <c r="D19" t="str">
-        <v>CAMPO BD</v>
-      </c>
-      <c r="E19" t="str">
-        <v>TIPO</v>
-      </c>
-      <c r="F19" t="str">
-        <v>CLAVE ÚNICA</v>
-      </c>
-      <c r="G19" t="str">
-        <v>REQUERIDO</v>
-      </c>
-      <c r="H19" t="str">
-        <v>DESTINO</v>
-      </c>
-      <c r="I19" t="str">
-        <v>NOTAS</v>
+        <v>Antes "STATUS DE CONTRATISTA". Columna BD: status_contratista. APROBADO / EN REVISIÓN / CON OBSERVACIONES / ANULADO</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Documentos</v>
+      </c>
+      <c r="B18">
+        <v>17</v>
+      </c>
+      <c r="C18" t="str">
+        <v>RESPONSABLE</v>
+      </c>
+      <c r="D18" t="str">
+        <v>responsable</v>
+      </c>
+      <c r="E18" t="str">
+        <v>texto</v>
+      </c>
+      <c r="F18" t="str">
+        <v/>
+      </c>
+      <c r="G18" t="str">
+        <v/>
+      </c>
+      <c r="H18" t="str">
+        <v>columna real</v>
+      </c>
+      <c r="I18" t="str">
+        <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Contratos</v>
-      </c>
-      <c r="B20">
-        <v>1</v>
+        <v>HOJA</v>
+      </c>
+      <c r="B20" t="str">
+        <v>ORDEN</v>
       </c>
       <c r="C20" t="str">
-        <v>CLASE CONTRATO</v>
+        <v>ENCABEZADO EN EXCEL</v>
       </c>
       <c r="D20" t="str">
-        <v>type</v>
+        <v>CAMPO BD</v>
       </c>
       <c r="E20" t="str">
-        <v>texto</v>
+        <v>TIPO</v>
       </c>
       <c r="F20" t="str">
-        <v/>
+        <v>CLAVE ÚNICA</v>
       </c>
       <c r="G20" t="str">
-        <v/>
+        <v>REQUERIDO</v>
       </c>
       <c r="H20" t="str">
-        <v>columna real</v>
+        <v>DESTINO</v>
       </c>
       <c r="I20" t="str">
-        <v/>
+        <v>NOTAS</v>
       </c>
     </row>
     <row r="21">
@@ -1184,13 +1187,13 @@
         <v>Contratos</v>
       </c>
       <c r="B21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C21" t="str">
-        <v>Tipo Inversion</v>
+        <v>CLASE CONTRATO</v>
       </c>
       <c r="D21" t="str">
-        <v>(extra_data)</v>
+        <v>type</v>
       </c>
       <c r="E21" t="str">
         <v>texto</v>
@@ -1202,7 +1205,7 @@
         <v/>
       </c>
       <c r="H21" t="str">
-        <v>extra_data (JSON)</v>
+        <v>columna real</v>
       </c>
       <c r="I21" t="str">
         <v/>
@@ -1213,10 +1216,10 @@
         <v>Contratos</v>
       </c>
       <c r="B22">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C22" t="str">
-        <v>Consultoria</v>
+        <v>Tipo Inversion</v>
       </c>
       <c r="D22" t="str">
         <v>(extra_data)</v>
@@ -1242,13 +1245,13 @@
         <v>Contratos</v>
       </c>
       <c r="B23">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C23" t="str">
-        <v>ESTADO</v>
+        <v>Consultoria</v>
       </c>
       <c r="D23" t="str">
-        <v>status</v>
+        <v>(extra_data)</v>
       </c>
       <c r="E23" t="str">
         <v>texto</v>
@@ -1260,7 +1263,7 @@
         <v/>
       </c>
       <c r="H23" t="str">
-        <v>columna real</v>
+        <v>extra_data (JSON)</v>
       </c>
       <c r="I23" t="str">
         <v/>
@@ -1271,13 +1274,13 @@
         <v>Contratos</v>
       </c>
       <c r="B24">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C24" t="str">
-        <v>A SAP Reg</v>
+        <v>ESTADO</v>
       </c>
       <c r="D24" t="str">
-        <v>(extra_data)</v>
+        <v>status</v>
       </c>
       <c r="E24" t="str">
         <v>texto</v>
@@ -1289,7 +1292,7 @@
         <v/>
       </c>
       <c r="H24" t="str">
-        <v>extra_data (JSON)</v>
+        <v>columna real</v>
       </c>
       <c r="I24" t="str">
         <v/>
@@ -1300,10 +1303,10 @@
         <v>Contratos</v>
       </c>
       <c r="B25">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C25" t="str">
-        <v>Estado Contrato SAP</v>
+        <v>A SAP Reg</v>
       </c>
       <c r="D25" t="str">
         <v>(extra_data)</v>
@@ -1329,10 +1332,10 @@
         <v>Contratos</v>
       </c>
       <c r="B26">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C26" t="str">
-        <v>B Custodia</v>
+        <v>Estado Contrato SAP</v>
       </c>
       <c r="D26" t="str">
         <v>(extra_data)</v>
@@ -1358,10 +1361,10 @@
         <v>Contratos</v>
       </c>
       <c r="B27">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C27" t="str">
-        <v>C OS(F=OK)</v>
+        <v>B Custodia</v>
       </c>
       <c r="D27" t="str">
         <v>(extra_data)</v>
@@ -1387,10 +1390,10 @@
         <v>Contratos</v>
       </c>
       <c r="B28">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C28" t="str">
-        <v>Estado OS SAP</v>
+        <v>C OS(F=OK)</v>
       </c>
       <c r="D28" t="str">
         <v>(extra_data)</v>
@@ -1416,10 +1419,10 @@
         <v>Contratos</v>
       </c>
       <c r="B29">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C29" t="str">
-        <v>RESPONSABLE</v>
+        <v>Estado OS SAP</v>
       </c>
       <c r="D29" t="str">
         <v>(extra_data)</v>
@@ -1445,10 +1448,10 @@
         <v>Contratos</v>
       </c>
       <c r="B30">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C30" t="str">
-        <v>GRUPO INVERSION</v>
+        <v>RESPONSABLE</v>
       </c>
       <c r="D30" t="str">
         <v>(extra_data)</v>
@@ -1474,10 +1477,10 @@
         <v>Contratos</v>
       </c>
       <c r="B31">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C31" t="str">
-        <v>AREA SOLICITANTE</v>
+        <v>GRUPO INVERSION</v>
       </c>
       <c r="D31" t="str">
         <v>(extra_data)</v>
@@ -1503,10 +1506,10 @@
         <v>Contratos</v>
       </c>
       <c r="B32">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C32" t="str">
-        <v>COD INVERSION</v>
+        <v>AREA SOLICITANTE</v>
       </c>
       <c r="D32" t="str">
         <v>(extra_data)</v>
@@ -1532,10 +1535,10 @@
         <v>Contratos</v>
       </c>
       <c r="B33">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C33" t="str">
-        <v>CC</v>
+        <v>COD INVERSION</v>
       </c>
       <c r="D33" t="str">
         <v>(extra_data)</v>
@@ -1561,10 +1564,10 @@
         <v>Contratos</v>
       </c>
       <c r="B34">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C34" t="str">
-        <v>CIRCUITO</v>
+        <v>CC</v>
       </c>
       <c r="D34" t="str">
         <v>(extra_data)</v>
@@ -1590,10 +1593,10 @@
         <v>Contratos</v>
       </c>
       <c r="B35">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C35" t="str">
-        <v>MODALIDAD CONTRATACION</v>
+        <v>CIRCUITO</v>
       </c>
       <c r="D35" t="str">
         <v>(extra_data)</v>
@@ -1619,10 +1622,10 @@
         <v>Contratos</v>
       </c>
       <c r="B36">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C36" t="str">
-        <v>Condiciones (Adel, % Ret FG, Ret FC)</v>
+        <v>MODALIDAD CONTRATACION</v>
       </c>
       <c r="D36" t="str">
         <v>(extra_data)</v>
@@ -1648,16 +1651,16 @@
         <v>Contratos</v>
       </c>
       <c r="B37">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C37" t="str">
-        <v>FECHA SUSCRIPCIÓN DE CONTRATO</v>
+        <v>Condiciones (Adel, % Ret FG, Ret FC)</v>
       </c>
       <c r="D37" t="str">
-        <v>start_date</v>
+        <v>(extra_data)</v>
       </c>
       <c r="E37" t="str">
-        <v>fecha</v>
+        <v>texto</v>
       </c>
       <c r="F37" t="str">
         <v/>
@@ -1666,7 +1669,7 @@
         <v/>
       </c>
       <c r="H37" t="str">
-        <v>columna real</v>
+        <v>extra_data (JSON)</v>
       </c>
       <c r="I37" t="str">
         <v/>
@@ -1677,13 +1680,13 @@
         <v>Contratos</v>
       </c>
       <c r="B38">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C38" t="str">
-        <v>FIN VIGENCIA CONTRATO</v>
+        <v>FECHA SUSCRIPCIÓN DE CONTRATO</v>
       </c>
       <c r="D38" t="str">
-        <v>end_date</v>
+        <v>start_date</v>
       </c>
       <c r="E38" t="str">
         <v>fecha</v>
@@ -1706,16 +1709,16 @@
         <v>Contratos</v>
       </c>
       <c r="B39">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C39" t="str">
-        <v>Fecha Acta de entrega de terreno</v>
+        <v>FIN VIGENCIA CONTRATO</v>
       </c>
       <c r="D39" t="str">
-        <v>(extra_data)</v>
+        <v>end_date</v>
       </c>
       <c r="E39" t="str">
-        <v>texto</v>
+        <v>fecha</v>
       </c>
       <c r="F39" t="str">
         <v/>
@@ -1724,7 +1727,7 @@
         <v/>
       </c>
       <c r="H39" t="str">
-        <v>extra_data (JSON)</v>
+        <v>columna real</v>
       </c>
       <c r="I39" t="str">
         <v/>
@@ -1735,10 +1738,10 @@
         <v>Contratos</v>
       </c>
       <c r="B40">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C40" t="str">
-        <v>Fecha Acta de INICIO DE OBRA2</v>
+        <v>Fecha Acta de entrega de terreno</v>
       </c>
       <c r="D40" t="str">
         <v>(extra_data)</v>
@@ -1764,10 +1767,10 @@
         <v>Contratos</v>
       </c>
       <c r="B41">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C41" t="str">
-        <v>PLAZO DE EJECUCION / FABRICACION</v>
+        <v>Fecha Acta de INICIO DE OBRA2</v>
       </c>
       <c r="D41" t="str">
         <v>(extra_data)</v>
@@ -1793,10 +1796,10 @@
         <v>Contratos</v>
       </c>
       <c r="B42">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C42" t="str">
-        <v>Fecha termino según contrato</v>
+        <v>PLAZO DE EJECUCION / FABRICACION</v>
       </c>
       <c r="D42" t="str">
         <v>(extra_data)</v>
@@ -1822,10 +1825,10 @@
         <v>Contratos</v>
       </c>
       <c r="B43">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C43" t="str">
-        <v>Z Ampliación de plazo</v>
+        <v>Fecha termino según contrato</v>
       </c>
       <c r="D43" t="str">
         <v>(extra_data)</v>
@@ -1851,10 +1854,10 @@
         <v>Contratos</v>
       </c>
       <c r="B44">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C44" t="str">
-        <v>Plazo penalizado</v>
+        <v>Z Ampliación de plazo</v>
       </c>
       <c r="D44" t="str">
         <v>(extra_data)</v>
@@ -1880,10 +1883,10 @@
         <v>Contratos</v>
       </c>
       <c r="B45">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C45" t="str">
-        <v>Plazo de Ejecucion ajustado</v>
+        <v>Plazo penalizado</v>
       </c>
       <c r="D45" t="str">
         <v>(extra_data)</v>
@@ -1909,10 +1912,10 @@
         <v>Contratos</v>
       </c>
       <c r="B46">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C46" t="str">
-        <v>Plazo total</v>
+        <v>Plazo de Ejecucion ajustado</v>
       </c>
       <c r="D46" t="str">
         <v>(extra_data)</v>
@@ -1938,10 +1941,10 @@
         <v>Contratos</v>
       </c>
       <c r="B47">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C47" t="str">
-        <v>Fecha Recepción Provisional / Fin según contrato (Ultima)</v>
+        <v>Plazo total</v>
       </c>
       <c r="D47" t="str">
         <v>(extra_data)</v>
@@ -1967,16 +1970,16 @@
         <v>Contratos</v>
       </c>
       <c r="B48">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C48" t="str">
-        <v>Fecha Recepcion Final</v>
+        <v>Fecha Recepción Provisional / Fin según contrato (Ultima)</v>
       </c>
       <c r="D48" t="str">
-        <v>actual_end_date</v>
+        <v>(extra_data)</v>
       </c>
       <c r="E48" t="str">
-        <v>fecha</v>
+        <v>texto</v>
       </c>
       <c r="F48" t="str">
         <v/>
@@ -1985,7 +1988,7 @@
         <v/>
       </c>
       <c r="H48" t="str">
-        <v>columna real</v>
+        <v>extra_data (JSON)</v>
       </c>
       <c r="I48" t="str">
         <v/>
@@ -1996,16 +1999,16 @@
         <v>Contratos</v>
       </c>
       <c r="B49">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C49" t="str">
-        <v>Plazo de garantia</v>
+        <v>Fecha Recepcion Final</v>
       </c>
       <c r="D49" t="str">
-        <v>(extra_data)</v>
+        <v>actual_end_date</v>
       </c>
       <c r="E49" t="str">
-        <v>texto</v>
+        <v>fecha</v>
       </c>
       <c r="F49" t="str">
         <v/>
@@ -2014,7 +2017,7 @@
         <v/>
       </c>
       <c r="H49" t="str">
-        <v>extra_data (JSON)</v>
+        <v>columna real</v>
       </c>
       <c r="I49" t="str">
         <v/>
@@ -2025,10 +2028,10 @@
         <v>Contratos</v>
       </c>
       <c r="B50">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C50" t="str">
-        <v>Inicio de operación del PYT</v>
+        <v>Plazo de garantia</v>
       </c>
       <c r="D50" t="str">
         <v>(extra_data)</v>
@@ -2054,10 +2057,10 @@
         <v>Contratos</v>
       </c>
       <c r="B51">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C51" t="str">
-        <v>Por Pagar Garantia (Cuenta 30 dias antes Venc.)</v>
+        <v>Inicio de operación del PYT</v>
       </c>
       <c r="D51" t="str">
         <v>(extra_data)</v>
@@ -2083,10 +2086,10 @@
         <v>Contratos</v>
       </c>
       <c r="B52">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C52" t="str">
-        <v>ID</v>
+        <v>Por Pagar Garantia (Cuenta 30 dias antes Venc.)</v>
       </c>
       <c r="D52" t="str">
         <v>(extra_data)</v>
@@ -2112,25 +2115,25 @@
         <v>Contratos</v>
       </c>
       <c r="B53">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C53" t="str">
-        <v>N° CONTRATO</v>
+        <v>ID</v>
       </c>
       <c r="D53" t="str">
-        <v>code</v>
+        <v>(extra_data)</v>
       </c>
       <c r="E53" t="str">
         <v>texto</v>
       </c>
       <c r="F53" t="str">
-        <v>SÍ</v>
+        <v/>
       </c>
       <c r="G53" t="str">
-        <v>SÍ</v>
+        <v/>
       </c>
       <c r="H53" t="str">
-        <v>columna real</v>
+        <v>extra_data (JSON)</v>
       </c>
       <c r="I53" t="str">
         <v/>
@@ -2141,25 +2144,25 @@
         <v>Contratos</v>
       </c>
       <c r="B54">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C54" t="str">
-        <v>CONTRATO DWH</v>
+        <v>N° CONTRATO</v>
       </c>
       <c r="D54" t="str">
-        <v>(extra_data)</v>
+        <v>code</v>
       </c>
       <c r="E54" t="str">
         <v>texto</v>
       </c>
       <c r="F54" t="str">
-        <v/>
+        <v>SÍ</v>
       </c>
       <c r="G54" t="str">
-        <v/>
+        <v>SÍ</v>
       </c>
       <c r="H54" t="str">
-        <v>extra_data (JSON)</v>
+        <v>columna real</v>
       </c>
       <c r="I54" t="str">
         <v/>
@@ -2170,10 +2173,10 @@
         <v>Contratos</v>
       </c>
       <c r="B55">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C55" t="str">
-        <v>ADENDA</v>
+        <v>CONTRATO DWH</v>
       </c>
       <c r="D55" t="str">
         <v>(extra_data)</v>
@@ -2199,10 +2202,10 @@
         <v>Contratos</v>
       </c>
       <c r="B56">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C56" t="str">
-        <v>RUC</v>
+        <v>ADENDA</v>
       </c>
       <c r="D56" t="str">
         <v>(extra_data)</v>
@@ -2228,10 +2231,10 @@
         <v>Contratos</v>
       </c>
       <c r="B57">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C57" t="str">
-        <v>EMPRESA</v>
+        <v>RUC</v>
       </c>
       <c r="D57" t="str">
         <v>(extra_data)</v>
@@ -2257,13 +2260,13 @@
         <v>Contratos</v>
       </c>
       <c r="B58">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C58" t="str">
-        <v>DESCRIPCION CONTRATO</v>
+        <v>EMPRESA</v>
       </c>
       <c r="D58" t="str">
-        <v>title</v>
+        <v>(extra_data)</v>
       </c>
       <c r="E58" t="str">
         <v>texto</v>
@@ -2272,10 +2275,10 @@
         <v/>
       </c>
       <c r="G58" t="str">
-        <v>SÍ</v>
+        <v/>
       </c>
       <c r="H58" t="str">
-        <v>columna real</v>
+        <v>extra_data (JSON)</v>
       </c>
       <c r="I58" t="str">
         <v/>
@@ -2286,13 +2289,13 @@
         <v>Contratos</v>
       </c>
       <c r="B59">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C59" t="str">
-        <v>Contrato en Chino</v>
+        <v>DESCRIPCION CONTRATO</v>
       </c>
       <c r="D59" t="str">
-        <v>(extra_data)</v>
+        <v>title</v>
       </c>
       <c r="E59" t="str">
         <v>texto</v>
@@ -2301,10 +2304,10 @@
         <v/>
       </c>
       <c r="G59" t="str">
-        <v/>
+        <v>SÍ</v>
       </c>
       <c r="H59" t="str">
-        <v>extra_data (JSON)</v>
+        <v>columna real</v>
       </c>
       <c r="I59" t="str">
         <v/>
@@ -2315,10 +2318,10 @@
         <v>Contratos</v>
       </c>
       <c r="B60">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C60" t="str">
-        <v>NOMBRE ESPECIFICO</v>
+        <v>Contrato en Chino</v>
       </c>
       <c r="D60" t="str">
         <v>(extra_data)</v>
@@ -2344,10 +2347,10 @@
         <v>Contratos</v>
       </c>
       <c r="B61">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C61" t="str">
-        <v>DESCRIPCION DE LA ADENDA</v>
+        <v>NOMBRE ESPECIFICO</v>
       </c>
       <c r="D61" t="str">
         <v>(extra_data)</v>
@@ -2373,10 +2376,10 @@
         <v>Contratos</v>
       </c>
       <c r="B62">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C62" t="str">
-        <v>CONTRATO_</v>
+        <v>DESCRIPCION DE LA ADENDA</v>
       </c>
       <c r="D62" t="str">
         <v>(extra_data)</v>
@@ -2402,10 +2405,10 @@
         <v>Contratos</v>
       </c>
       <c r="B63">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C63" t="str">
-        <v>EMPRESA_</v>
+        <v>CONTRATO_</v>
       </c>
       <c r="D63" t="str">
         <v>(extra_data)</v>
@@ -2431,10 +2434,10 @@
         <v>Contratos</v>
       </c>
       <c r="B64">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C64" t="str">
-        <v>CONTRATO_ NOMBRE INFORME</v>
+        <v>EMPRESA_</v>
       </c>
       <c r="D64" t="str">
         <v>(extra_data)</v>
@@ -2460,13 +2463,13 @@
         <v>Contratos</v>
       </c>
       <c r="B65">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C65" t="str">
-        <v>MONEDA</v>
+        <v>CONTRATO_ NOMBRE INFORME</v>
       </c>
       <c r="D65" t="str">
-        <v>currency</v>
+        <v>(extra_data)</v>
       </c>
       <c r="E65" t="str">
         <v>texto</v>
@@ -2478,7 +2481,7 @@
         <v/>
       </c>
       <c r="H65" t="str">
-        <v>columna real</v>
+        <v>extra_data (JSON)</v>
       </c>
       <c r="I65" t="str">
         <v/>
@@ -2489,16 +2492,16 @@
         <v>Contratos</v>
       </c>
       <c r="B66">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C66" t="str">
-        <v>PPTO BASE</v>
+        <v>MONEDA</v>
       </c>
       <c r="D66" t="str">
-        <v>(extra_data)</v>
+        <v>currency</v>
       </c>
       <c r="E66" t="str">
-        <v>numero</v>
+        <v>texto</v>
       </c>
       <c r="F66" t="str">
         <v/>
@@ -2507,7 +2510,7 @@
         <v/>
       </c>
       <c r="H66" t="str">
-        <v>extra_data (JSON)</v>
+        <v>columna real</v>
       </c>
       <c r="I66" t="str">
         <v/>
@@ -2518,10 +2521,10 @@
         <v>Contratos</v>
       </c>
       <c r="B67">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C67" t="str">
-        <v>MONTO CONTRATADO S/ (SIN IGV)</v>
+        <v>PPTO BASE</v>
       </c>
       <c r="D67" t="str">
         <v>(extra_data)</v>
@@ -2547,10 +2550,10 @@
         <v>Contratos</v>
       </c>
       <c r="B68">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C68" t="str">
-        <v>MONTO CONTRATADO US$ (SIN IGV)</v>
+        <v>MONTO CONTRATADO S/ (SIN IGV)</v>
       </c>
       <c r="D68" t="str">
         <v>(extra_data)</v>
@@ -2576,10 +2579,10 @@
         <v>Contratos</v>
       </c>
       <c r="B69">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C69" t="str">
-        <v>MONTO CONTRATADO S/ (CON IGV)</v>
+        <v>MONTO CONTRATADO US$ (SIN IGV)</v>
       </c>
       <c r="D69" t="str">
         <v>(extra_data)</v>
@@ -2605,10 +2608,10 @@
         <v>Contratos</v>
       </c>
       <c r="B70">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C70" t="str">
-        <v>MONTO CONTRATADO US$ (CON IGV)</v>
+        <v>MONTO CONTRATADO S/ (CON IGV)</v>
       </c>
       <c r="D70" t="str">
         <v>(extra_data)</v>
@@ -2629,9 +2632,38 @@
         <v/>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>Contratos</v>
+      </c>
+      <c r="B71">
+        <v>51</v>
+      </c>
+      <c r="C71" t="str">
+        <v>MONTO CONTRATADO US$ (CON IGV)</v>
+      </c>
+      <c r="D71" t="str">
+        <v>(extra_data)</v>
+      </c>
+      <c r="E71" t="str">
+        <v>numero</v>
+      </c>
+      <c r="F71" t="str">
+        <v/>
+      </c>
+      <c r="G71" t="str">
+        <v/>
+      </c>
+      <c r="H71" t="str">
+        <v>extra_data (JSON)</v>
+      </c>
+      <c r="I71" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I70"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I71"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>